<commit_message>
big update for khkt
</commit_message>
<xml_diff>
--- a/design-stitch/Template.xlsx
+++ b/design-stitch/Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Web\viviora\design-stitch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A85E32A-A613-4D89-B021-3A3C4C901421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5931FE2A-3C03-4D88-83AF-8BE6C064537B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-24" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Type</t>
   </si>
@@ -58,6 +58,15 @@
   </si>
   <si>
     <t>Option 2/False</t>
+  </si>
+  <si>
+    <t>TF</t>
+  </si>
+  <si>
+    <t>1+2=1</t>
+  </si>
+  <si>
+    <t>*</t>
   </si>
 </sst>
 </file>
@@ -381,7 +390,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="14.7109375" customWidth="1"/>
@@ -434,6 +443,17 @@
         <v>8</v>
       </c>
     </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>